<commit_message>
Import: update only changed rows (shows unchanged), empty cell clears the saved value
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019x7omn2dFBF8qLBo7dKqKg
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -678,7 +678,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>3. Link tables by slug/name, never by ID. Same slug as in the database = update, new slug = create. Nothing is deleted.</t>
+          <t>3. Link tables by slug/name, never by ID. New slug = create. Same slug = update, but only if a value changed (identical rows are skipped). Nothing is deleted.</t>
         </is>
       </c>
       <c r="B6" s="2" t="n"/>
@@ -696,7 +696,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>5. Dates YYYY-MM-DD. Yes/No columns use 1 or 0. An empty cell keeps the value already saved. Images/icons cannot be uploaded here (add them in Admin afterwards).</t>
+          <t>5. Dates YYYY-MM-DD. Yes/No columns use 1 or 0. An EMPTY CELL CLEARS the saved value (columns that can never be empty, such as name, line_type or sort_order, keep their value). Delete a whole column to leave its values untouched. Images/icons cannot be uploaded here (add them in Admin afterwards).</t>
         </is>
       </c>
       <c r="B8" s="2" t="n"/>

</xml_diff>

<commit_message>
Import: facilities can list their nearby exits (exits column), compared and synced like other fields
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019x7omn2dFBF8qLBo7dKqKg
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -825,7 +825,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Order 7. floor_name must exist in floors for that station. location_type: inside/outside.</t>
+          <t>Order 7. floor_name must exist in floors for that station. exits = nearby exits of this facility, exit names from the exits sheet separated by ; (empty cell clears them). note is a separate column. location_type: inside/outside.</t>
         </is>
       </c>
     </row>
@@ -1785,13 +1785,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
@@ -1816,25 +1816,30 @@
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
+          <t>exits</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
           <t>facility_count</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>note_japanese</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>location_type</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>sort_order</t>
         </is>
@@ -1856,25 +1861,30 @@
           <t>elevator</t>
         </is>
       </c>
-      <c r="D2" s="6" t="n">
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>North Exit; South Exit</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Near the north gate</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>北改札の近く</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>inside</t>
         </is>
       </c>
-      <c r="H2" s="6" t="n">
+      <c r="I2" s="6" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Bulk import: station region + stat cards, facility category, platform map group; updated Excel template
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -628,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -889,6 +889,41 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>New columns (all optional - delete the column to leave stored values untouched):</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>facilities: category = storage, tickets, access, shops, transport or other (groups the 'At this station' chips). Blank keeps the stored value ('other' for new rows).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>floor_facilities: 'exits' = nearby exit names separated by | (exit names must exist in the exits sheet).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -900,7 +935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -912,6 +947,8 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -960,6 +997,16 @@
           <t>sort_order</t>
         </is>
       </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>platform_group</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>platform_group_japanese</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -996,6 +1043,16 @@
       <c r="H2" s="6" t="inlineStr"/>
       <c r="I2" s="6" t="n">
         <v>1</v>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>Deep underground</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>地下深部</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1460,7 +1517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1473,6 +1530,16 @@
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="32" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="28" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1526,6 +1593,56 @@
           <t>verified_at</t>
         </is>
       </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>region_japanese</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>stat_lines_note</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>stat_lines_note_japanese</t>
+        </is>
+      </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>stat_riders_value</t>
+        </is>
+      </c>
+      <c r="P1" s="5" t="inlineStr">
+        <is>
+          <t>stat_riders_note</t>
+        </is>
+      </c>
+      <c r="Q1" s="5" t="inlineStr">
+        <is>
+          <t>stat_riders_note_japanese</t>
+        </is>
+      </c>
+      <c r="R1" s="5" t="inlineStr">
+        <is>
+          <t>stat_opened_value</t>
+        </is>
+      </c>
+      <c r="S1" s="5" t="inlineStr">
+        <is>
+          <t>stat_opened_note</t>
+        </is>
+      </c>
+      <c r="T1" s="5" t="inlineStr">
+        <is>
+          <t>stat_opened_note_japanese</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -1576,6 +1693,56 @@
       <c r="J2" s="6" t="inlineStr">
         <is>
           <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>Chiyoda City · Tokyo</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>東京都千代田区</t>
+        </is>
+      </c>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
+          <t>22 JR lines + Tokyo Metro Marunouchi Line</t>
+        </is>
+      </c>
+      <c r="N2" s="6" t="inlineStr">
+        <is>
+          <t>JR22路線＋東京メトロ丸ノ内線</t>
+        </is>
+      </c>
+      <c r="O2" s="6" t="inlineStr">
+        <is>
+          <t>434,564 / day</t>
+        </is>
+      </c>
+      <c r="P2" s="6" t="inlineStr">
+        <is>
+          <t>JR East boarding passengers, FY2024</t>
+        </is>
+      </c>
+      <c r="Q2" s="6" t="inlineStr">
+        <is>
+          <t>JR東日本の乗車人員（2024年度）</t>
+        </is>
+      </c>
+      <c r="R2" s="6" t="inlineStr">
+        <is>
+          <t>1914</t>
+        </is>
+      </c>
+      <c r="S2" s="6" t="inlineStr">
+        <is>
+          <t>Opened (Marunouchi building)</t>
+        </is>
+      </c>
+      <c r="T2" s="6" t="inlineStr">
+        <is>
+          <t>開業（丸の内駅舎）</t>
         </is>
       </c>
     </row>
@@ -1659,13 +1826,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1689,6 +1857,11 @@
           <t>sort_order</t>
         </is>
       </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -1708,6 +1881,11 @@
       </c>
       <c r="D2" s="6" t="n">
         <v>1</v>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>access</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Station page: Overview with facts card (opened, operators, address, codes, riders, map); station address field + import column
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -889,6 +889,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
@@ -899,7 +900,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:V2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1540,6 +1541,8 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="28" customWidth="1" min="19" max="19"/>
     <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="30" customWidth="1" min="21" max="21"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1643,6 +1646,16 @@
           <t>stat_opened_note_japanese</t>
         </is>
       </c>
+      <c r="U1" s="5" t="inlineStr">
+        <is>
+          <t>address</t>
+        </is>
+      </c>
+      <c r="V1" s="5" t="inlineStr">
+        <is>
+          <t>address_japanese</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -1743,6 +1756,16 @@
       <c r="T2" s="6" t="inlineStr">
         <is>
           <t>開業（丸の内駅舎）</t>
+        </is>
+      </c>
+      <c r="U2" s="6" t="inlineStr">
+        <is>
+          <t>1-6-5 Marunouchi, Chiyoda City</t>
+        </is>
+      </c>
+      <c r="V2" s="6" t="inlineStr">
+        <is>
+          <t>千代田区丸の内1-6-5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bulk import: sides sheet + sides_note columns; template updated
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -17,8 +17,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="floor_facilities" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exits" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="platforms" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sides" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -628,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -862,7 +863,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>top_picks</t>
+          <t>sides</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -870,14 +871,14 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Order 10. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+          <t>Order 10. Key: station_slug + name. One row per side of a station (e.g. Marunouchi / Yaesu): red subtitle + description. The crossing note is the stations column sides_note.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>station_top_picks</t>
+          <t>top_picks</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
@@ -885,43 +886,67 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Order 11. location_type: inside/outside/inside_outside.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
+          <t>Order 11. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>station_top_picks</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Order 12. location_type: inside/outside/inside_outside.</t>
+        </is>
+      </c>
+    </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="3" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>New columns (all optional - delete the column to leave stored values untouched):</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>facilities: category = storage, tickets, access, shops, transport or other (groups the 'At this station' chips). Blank keeps the stored value ('other' for new rows).</t>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
+          <t>facilities: category = storage, tickets, access, shops, transport or other (groups the 'At this station' chips). Blank keeps the stored value ('other' for new rows).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>floor_facilities: 'exits' = nearby exit names separated by | (exit names must exist in the exits sheet).</t>
+          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
         </is>
       </c>
     </row>
@@ -1068,6 +1093,112 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>name_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>subtitle</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>subtitle_japanese</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>description_japanese</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#tokyo</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Marunouchi side</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>丸の内</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>West side · Red-brick historic front</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>西側・赤レンガの駅舎</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Faces the Imperial Palace. The 1914 red-brick station building stands here, with The Tokyo Station Hotel inside.</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>皇居に面しています。1914年の赤レンガ駅舎があります。</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1209,7 +1340,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1518,7 +1649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:X2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1543,6 +1674,8 @@
     <col width="20" customWidth="1" min="20" max="20"/>
     <col width="30" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="44" customWidth="1" min="23" max="23"/>
+    <col width="36" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1656,6 +1789,16 @@
           <t>address_japanese</t>
         </is>
       </c>
+      <c r="W1" s="5" t="inlineStr">
+        <is>
+          <t>sides_note</t>
+        </is>
+      </c>
+      <c r="X1" s="5" t="inlineStr">
+        <is>
+          <t>sides_note_japanese</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -1766,6 +1909,16 @@
       <c r="V2" s="6" t="inlineStr">
         <is>
           <t>千代田区丸の内1-6-5</t>
+        </is>
+      </c>
+      <c r="W2" s="6" t="inlineStr">
+        <is>
+          <t>To cross between the west and east sides without a ticket, use the free passage at the north end.</t>
+        </is>
+      </c>
+      <c r="X2" s="6" t="inlineStr">
+        <is>
+          <t>改札を通らずに東西を行き来するには、北端の自由通路をご利用ください。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bulk import never creates, changes or deletes facilities; template drops the facilities sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -12,14 +12,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lines" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stations" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="line_stations" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="facilities" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="floors" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="floor_facilities" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exits" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="platforms" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sides" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="floors" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="floor_facilities" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exits" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="platforms" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sides" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -198,21 +197,6 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Order 10. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment11.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Template</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
         <t>Order 11. location_type: inside/outside/inside_outside.</t>
       </text>
     </comment>
@@ -273,21 +257,6 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Order 5. Icons cannot be uploaded in Excel; add them in Admin &gt; Facilities.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Template</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
         <t>Order 6. Key: station_slug + name.</t>
       </text>
     </comment>
@@ -295,7 +264,7 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Template</author>
@@ -310,7 +279,7 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Template</author>
@@ -325,6 +294,21 @@
 </comments>
 </file>
 
+<file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Template</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Order 9. Key: station_slug + platform_number + line_slug. line_slug and floor_name are optional.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/comments/comment9.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
@@ -333,7 +317,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Order 9. Key: station_slug + platform_number + line_slug. line_slug and floor_name are optional.</t>
+        <t>Order 10. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
       </text>
     </comment>
   </commentList>
@@ -788,7 +772,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>facilities</t>
+          <t>floors</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
@@ -796,14 +780,14 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Order 5. Icons cannot be uploaded in Excel; add them in Admin &gt; Facilities.</t>
+          <t>Order 5. Key: station_slug + name.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>floors</t>
+          <t>floor_facilities</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -811,14 +795,14 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Order 6. Key: station_slug + name.</t>
+          <t>Order 6. floor_name must exist in floors for that station. exits = nearby exits of this facility, exit names from the exits sheet separated by ; (empty cell clears them). note is a separate column. location_type: inside/outside. facility_slug must already exist in Admin &gt; Facilities (the importer never creates or changes facilities).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>floor_facilities</t>
+          <t>exits</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
@@ -826,14 +810,14 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Order 7. floor_name must exist in floors for that station. exits = nearby exits of this facility, exit names from the exits sheet separated by ; (empty cell clears them). note is a separate column. location_type: inside/outside.</t>
+          <t>Order 7. Key: station_slug + name.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>exits</t>
+          <t>platforms</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -841,14 +825,14 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Order 8. Key: station_slug + name.</t>
+          <t>Order 8. Key: station_slug + platform_number + line_slug. line_slug and floor_name are optional.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>platforms</t>
+          <t>sides</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
@@ -856,14 +840,14 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Order 9. Key: station_slug + platform_number + line_slug. line_slug and floor_name are optional.</t>
+          <t>Order 9. Key: station_slug + name. One row per side of a station (e.g. Marunouchi / Yaesu): red subtitle + description. The crossing note is the stations column sides_note.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>sides</t>
+          <t>top_picks</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -871,14 +855,14 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Order 10. Key: station_slug + name. One row per side of a station (e.g. Marunouchi / Yaesu): red subtitle + description. The crossing note is the stations column sides_note.</t>
+          <t>Order 10. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>top_picks</t>
+          <t>station_top_picks</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
@@ -886,69 +870,59 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Order 11. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+          <t>Order 11. location_type: inside/outside/inside_outside.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>station_top_picks</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Order 12. location_type: inside/outside/inside_outside.</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n"/>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>New columns (all optional - delete the column to leave stored values untouched):</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>New columns (all optional - delete the column to leave stored values untouched):</t>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
+          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>facilities: category = storage, tickets, access, shops, transport or other (groups the 'At this station' chips). Blank keeps the stored value ('other' for new rows).</t>
+          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
+          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
+          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
-        </is>
-      </c>
+      <c r="A29" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -956,138 +930,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="27" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>station_slug</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>platform_number</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>line_slug</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>floor_name</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>destinations</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>destinations_japanese</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>notes_japanese</t>
-        </is>
-      </c>
-      <c r="I1" s="5" t="inlineStr">
-        <is>
-          <t>sort_order</t>
-        </is>
-      </c>
-      <c r="J1" s="5" t="inlineStr">
-        <is>
-          <t>platform_group</t>
-        </is>
-      </c>
-      <c r="K1" s="5" t="inlineStr">
-        <is>
-          <t>platform_group_japanese</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>#nishi-nippori</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>yamanote</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>2F</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>Ueno, Tokyo</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>上野・東京方面</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr"/>
-      <c r="H2" s="6" t="inlineStr"/>
-      <c r="I2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" s="6" t="inlineStr">
-        <is>
-          <t>Deep underground</t>
-        </is>
-      </c>
-      <c r="K2" s="6" t="inlineStr">
-        <is>
-          <t>地下深部</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1193,7 +1035,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1340,7 +1182,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2002,80 +1844,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>slug</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>name_japanese</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>sort_order</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>#elevator</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>Elevator</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>エレベーター</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>access</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2133,7 +1901,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2253,7 +2021,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2369,4 +2137,136 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>platform_number</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>line_slug</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>floor_name</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>destinations</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>destinations_japanese</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>notes_japanese</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>platform_group</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>platform_group_japanese</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#nishi-nippori</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>yamanote</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>2F</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Ueno, Tokyo</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>上野・東京方面</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr"/>
+      <c r="H2" s="6" t="inlineStr"/>
+      <c r="I2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>Deep underground</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>地下深部</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Station page: Getting there table + Manage Routes admin + routes import sheet; template updated
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -17,8 +17,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exits" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="platforms" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sides" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="routes" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -613,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -847,7 +848,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>top_picks</t>
+          <t>routes</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -855,14 +856,14 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Order 10. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+          <t>Order 10. Key: station_slug + from_place + route. One row per way of getting to the station ("Getting there" table). The footnote is the stations column routes_note.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>station_top_picks</t>
+          <t>top_picks</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
@@ -870,59 +871,79 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Order 11. location_type: inside/outside/inside_outside.</t>
+          <t>Order 11. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n"/>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
+      <c r="B22" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Order 12. location_type: inside/outside/inside_outside.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>New columns (all optional - delete the column to leave stored values untouched):</t>
-        </is>
-      </c>
+      <c r="A23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
+          <t>station_top_picks</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>New columns (all optional - delete the column to leave stored values untouched):</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
+          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="n"/>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1036,6 +1057,134 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>from_place</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>from_place_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>route_japanese</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>travel_time</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>travel_time_japanese</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>cost_japanese</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#tokyo</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Narita Airport</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>成田空港</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Narita Express (N'EX), direct to the underground Sobu/Yokosuka platforms</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>成田エクスプレス（N'EX）で東京駅の地下ホームへ直通</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>≈ 53 min</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>約53分</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>¥3,140</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>3,140円</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1182,7 +1331,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1491,7 +1640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:Z2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1518,6 +1667,8 @@
     <col width="22" customWidth="1" min="22" max="22"/>
     <col width="44" customWidth="1" min="23" max="23"/>
     <col width="36" customWidth="1" min="24" max="24"/>
+    <col width="44" customWidth="1" min="25" max="25"/>
+    <col width="36" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1641,6 +1792,16 @@
           <t>sides_note_japanese</t>
         </is>
       </c>
+      <c r="Y1" s="5" t="inlineStr">
+        <is>
+          <t>routes_note</t>
+        </is>
+      </c>
+      <c r="Z1" s="5" t="inlineStr">
+        <is>
+          <t>routes_note_japanese</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -1761,6 +1922,16 @@
       <c r="X2" s="6" t="inlineStr">
         <is>
           <t>改札を通らずに東西を行き来するには、北端の自由通路をご利用ください。</t>
+        </is>
+      </c>
+      <c r="Y2" s="6" t="inlineStr">
+        <is>
+          <t>Fares and times as published by the operators; check before you travel.</t>
+        </is>
+      </c>
+      <c r="Z2" s="6" t="inlineStr">
+        <is>
+          <t>運賃・所要時間は各社の公表値です。ご利用前にご確認ください。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Station page: Exits & station tips (exits table, exit photos, tips); admin Exit photos & tips; tips import sheet; demo/template updated
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -18,8 +18,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="platforms" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sides" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="routes" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tips" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -614,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -863,7 +864,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>top_picks</t>
+          <t>tips</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
@@ -871,77 +872,99 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Order 11. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+          <t>Order 11. Key: station_slug + tip. One row per bullet under "Exits &amp; station tips". Exit photos are uploaded in Admin (Exit photos &amp; tips); the table above them comes from the exits sheet (name + description).</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>top_picks</t>
+        </is>
+      </c>
       <c r="B22" s="2" t="n">
         <v>12</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Order 12. location_type: inside/outside/inside_outside.</t>
+          <t>Order 12. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n"/>
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Order 13. location_type: inside/outside/inside_outside.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>station_top_picks</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>New columns (all optional - delete the column to leave stored values untouched):</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
+          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
+          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
+          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
+          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
           <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are uploaded in Admin &gt; Stations &gt; Exit photos &amp; tips.</t>
         </is>
       </c>
     </row>
@@ -1190,6 +1213,68 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>tip</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>tip_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#tokyo</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>The Marunouchi Central gate is IC card only and open 9:30-17:00; use the North or South gates with a paper ticket.</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>丸の内中央口はIC専用（9:30〜17:00）。紙のきっぷは北口・南口へ。</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1331,7 +1416,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1640,7 +1725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:AB2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1669,6 +1754,8 @@
     <col width="36" customWidth="1" min="24" max="24"/>
     <col width="44" customWidth="1" min="25" max="25"/>
     <col width="36" customWidth="1" min="26" max="26"/>
+    <col width="44" customWidth="1" min="27" max="27"/>
+    <col width="36" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1802,6 +1889,16 @@
           <t>routes_note_japanese</t>
         </is>
       </c>
+      <c r="AA1" s="5" t="inlineStr">
+        <is>
+          <t>exits_note</t>
+        </is>
+      </c>
+      <c r="AB1" s="5" t="inlineStr">
+        <is>
+          <t>exits_note_japanese</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -1932,6 +2029,16 @@
       <c r="Z2" s="6" t="inlineStr">
         <is>
           <t>運賃・所要時間は各社の公表値です。ご利用前にご確認ください。</t>
+        </is>
+      </c>
+      <c r="AA2" s="6" t="inlineStr">
+        <is>
+          <t>Signs inside the station say "Exit", signs outside say "Entrance". They are the same places.</t>
+        </is>
+      </c>
+      <c r="AB2" s="6" t="inlineStr">
+        <is>
+          <t>駅構内の表示は「出口」、駅外の表示は「入口」ですが、同じ場所です。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Exit photos belong to each exit (upload in Manage Exits, works for imported exits); photo_caption import columns; template/demo updated
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -872,7 +872,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Order 11. Key: station_slug + tip. One row per bullet under "Exits &amp; station tips". Exit photos are uploaded in Admin (Exit photos &amp; tips); the table above them comes from the exits sheet (name + description).</t>
+          <t>Order 11. Key: station_slug + tip. One row per bullet under "Exits &amp; station tips". Exit photos are uploaded in Admin &gt; Manage Exits; the table above them comes from the exits sheet (name + description).</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,11 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>station_top_picks</t>
+        </is>
+      </c>
       <c r="B23" s="2" t="n">
         <v>13</v>
       </c>
@@ -906,11 +910,7 @@
       <c r="A24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>station_top_picks</t>
-        </is>
-      </c>
+      <c r="A25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -964,7 +964,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are uploaded in Admin &gt; Stations &gt; Exit photos &amp; tips.</t>
+          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2317,6 +2317,8 @@
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2365,6 +2367,16 @@
           <t>sort_order</t>
         </is>
       </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>photo_caption</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>photo_caption_japanese</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -2409,6 +2421,16 @@
       </c>
       <c r="I2" s="6" t="n">
         <v>1</v>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>What you see on leaving: the white KITTE building, straight across the crossing.</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>出口を出ると：目の前にKITTEの白いビルが見えます。</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Station page: When to visit seasons section (table, admin page, importer, template)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -19,8 +19,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sides" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="routes" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tips" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="seasons" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -90,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -100,6 +101,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -615,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -879,7 +883,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>top_picks</t>
+          <t>seasons</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -887,14 +891,14 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Order 12. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+          <t>Order 12. Key: station_slug + season. season: spring/summer/autumn/winter (one row each). One row per season of "When to visit": months (red label, e.g. Mar – May) + description.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>station_top_picks</t>
+          <t>top_picks</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
@@ -902,12 +906,24 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Order 13. location_type: inside/outside/inside_outside.</t>
+          <t>Order 13. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>station_top_picks</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Order 14. location_type: inside/outside/inside_outside.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
@@ -968,6 +984,38 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1275,6 +1323,92 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>season</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>months_japanese</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>description_japanese</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>#tokyo</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>spring</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Mar – May</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>3月〜5月</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Cherry blossoms around Chidorigafuchi, by the Imperial Palace moat, usually peak in late March to early April.</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>千鳥ケ淵の桜は例年3月下旬から4月上旬が見頃です。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1416,7 +1550,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Station page: Practical tips and FAQ sections (tables, admin pages, importer, template)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -20,8 +20,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="routes" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tips" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="seasons" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="practical_tips" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="faqs" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -619,7 +621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -898,7 +900,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>top_picks</t>
+          <t>practical_tips</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
@@ -906,14 +908,14 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Order 13. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+          <t>Order 13. Key: station_slug + tip. One row per bullet under "Practical tips".</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>station_top_picks</t>
+          <t>faqs</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -921,101 +923,112 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Order 14. location_type: inside/outside/inside_outside.</t>
+          <t>Order 14. Key: station_slug + question. One row per FAQ (question + answer, opens when clicked).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>top_picks</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Order 15. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>station_top_picks</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Order 16. location_type: inside/outside/inside_outside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>New columns (all optional - delete the column to leave stored values untouched):</t>
         </is>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
-        </is>
-      </c>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
+          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
+          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
+          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
+          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
+          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
           <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
         </is>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>practical_tips: bullets under 'Practical tips'. faqs: 'FAQ' list; answer is required. Both are also editable in Admin &gt; Stations &gt; Practical tips / FAQs.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1409,6 +1422,160 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>tip</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>tip_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>#tokyo</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>The Tokaido-Sanyo Shinkansen (JR Central) uses platforms 14–19 and blue gates; the Tohoku, Joetsu and Hokuriku Shinkansen (JR East) use platforms 20–23 and green gates. Check which colour your train belongs to before you follow the signs.</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>東海道・山陽新幹線は14〜19番線（青い改札）、東北・上越・北陸新幹線は20〜23番線（緑の改札）です。</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>question</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>question_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>answer</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>answer_japanese</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>#tokyo</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Where are the coin lockers at Tokyo Station?</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>コインロッカーはどこ？</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Lockers are near the Marunouchi and Yaesu gates, but they fill up quickly on weekdays. Use the locker search/reserve QR code or a staffed luggage counter.</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>丸の内口と八重洲口の改札付近にありますが、平日は早く埋まります。</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1550,7 +1717,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Station page: Day trips section with photos; station list actions trimmed to Edit/Delete
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -22,8 +22,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="seasons" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="practical_tips" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="faqs" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="day_trips" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -621,7 +622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -930,7 +931,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>top_picks</t>
+          <t>day_trips</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
@@ -938,14 +939,14 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Order 15. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+          <t>Order 15. Key: station_slug + name. One row per place under "Day trips": travel_time (e.g. ≈ 25–40 min) · transport (e.g. JR lines, direct), description, map_url (the Map button). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Day trips.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>station_top_picks</t>
+          <t>top_picks</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -953,82 +954,105 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Order 16. location_type: inside/outside/inside_outside.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+          <t>Order 16. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>station_top_picks</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Order 17. location_type: inside/outside/inside_outside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>New columns (all optional - delete the column to leave stored values untouched):</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
-        </is>
-      </c>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
+          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
+          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
+          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
+          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
+          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
+          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
+          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
           <t>practical_tips: bullets under 'Practical tips'. faqs: 'FAQ' list; answer is required. Both are also editable in Admin &gt; Stations &gt; Practical tips / FAQs.</t>
         </is>
       </c>
     </row>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1580,6 +1604,145 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>name_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>travel_time</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>travel_time_japanese</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>transport_japanese</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>description_japanese</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>map_url</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>#tokyo</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Yokohama</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>横浜</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>≈ 25–40 min</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>約25〜40分</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>JR lines, direct</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>JR線・乗換なし</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>GO TOKYO lists 25–40 minutes from Tokyo Station to Yokohama Station on JR lines; Yokohama's official visitors guide names the JR Tokaido, Yokosuka and Keihin-Tohoku lines.</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>東京駅から横浜駅までJR線で約25〜40分。東海道線・横須賀線・京浜東北線が利用できます。</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Yokohama+Station</t>
+        </is>
+      </c>
+      <c r="K2" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -1717,7 +1880,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Station page: Facilities section (table + photo cards), admin guide page, importer, template
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -23,8 +23,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="practical_tips" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="faqs" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="day_trips" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="facility_guide" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -946,7 +947,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>top_picks</t>
+          <t>facility_guide</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -954,14 +955,14 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Order 16. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+          <t>Order 16. Key: station_slug + name. The public "Facilities" section (not the facility icons of the floor map): a row with a description is listed in the table (Facility / Where and what to know); a row with a photo also gets a photo card (name + photo_caption). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Facilities guide.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>station_top_picks</t>
+          <t>top_picks</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
@@ -969,84 +970,98 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Order 17. location_type: inside/outside/inside_outside.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28"/>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+          <t>Order 17. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>station_top_picks</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Order 18. location_type: inside/outside/inside_outside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>New columns (all optional - delete the column to leave stored values untouched):</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
-        </is>
-      </c>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
+          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
+          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
+          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
+          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
+          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
+          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
+          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
           <t>practical_tips: bullets under 'Practical tips'. faqs: 'FAQ' list; answer is required. Both are also editable in Admin &gt; Stations &gt; Practical tips / FAQs.</t>
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40"/>
     <row r="41"/>
     <row r="42"/>
@@ -1739,6 +1754,105 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>name_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>description_japanese</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>photo_caption</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>photo_caption_japanese</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>#tokyo</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Coin lockers</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>コインロッカー</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>The locker banks we checked near the Marunouchi gates on 8 October 2026 cost ¥500 (S), ¥700 (M) and ¥900 (L). All are 34 cm wide and 65 cm deep; the height is 33 cm (S), 50 cm (M) or 86 cm (L). The ma…</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr"/>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>From ¥500. This bank takes IC card, credit card or QR payment, not cash.</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr"/>
+      <c r="H2" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1880,7 +1994,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Station page: Buses & taxis section (table + photo cards), admin page, importer, template
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -24,8 +24,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="faqs" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="day_trips" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="facility_guide" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="buses_taxis" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -962,7 +963,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>top_picks</t>
+          <t>buses_taxis</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
@@ -970,14 +971,14 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Order 17. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+          <t>Order 17. Key: station_slug + place. The public "Buses &amp; taxis" section: a row with service or notes is listed in the table (Where / Service / Notes); a row with a photo also gets a photo card (photo_title, or place, + photo_caption). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Buses &amp; taxis.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>station_top_picks</t>
+          <t>top_picks</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -985,84 +986,98 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Order 18. location_type: inside/outside/inside_outside.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29"/>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+          <t>Order 18. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>station_top_picks</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Order 19. location_type: inside/outside/inside_outside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>New columns (all optional - delete the column to leave stored values untouched):</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
-        </is>
-      </c>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
+          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
+          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
+          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
+          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
+          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
+          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
+          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
           <t>practical_tips: bullets under 'Practical tips'. faqs: 'FAQ' list; answer is required. Both are also editable in Admin &gt; Stations &gt; Practical tips / FAQs.</t>
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41"/>
     <row r="42"/>
     <row r="43"/>
@@ -1853,6 +1868,140 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>place_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>service</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>service_japanese</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>notes_japanese</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>photo_title</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>photo_title_japanese</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>photo_caption</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>photo_caption_japanese</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>#tokyo</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Marunouchi North Exit</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>丸の内北口</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Toei Bus: Higashi 43 (for Arakawa-dote)</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>都営バス 東43（荒川土手行）</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>City bus stops on the Marunouchi side</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>丸の内側のバス停</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr"/>
+      <c r="I2" s="7" t="inlineStr"/>
+      <c r="J2" s="7" t="inlineStr"/>
+      <c r="K2" s="7" t="inlineStr"/>
+      <c r="L2" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1987,83 +2136,6 @@
   <dataValidations count="1">
     <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"landmark,food,shopping,museum,park,temple"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>station_slug</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>top_pick_slug</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>walking_minutes</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>location_type</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>sort_order</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>#nishi-nippori</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>asakura-museum</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>outside</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"inside,outside,inside_outside"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2153,6 +2225,83 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>top_pick_slug</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>walking_minutes</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>location_type</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#nishi-nippori</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>asakura-museum</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>outside</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"inside,outside,inside_outside"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>

<commit_message>
Station page: Things to do section, admin page, importer, template
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -25,8 +25,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="day_trips" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="facility_guide" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="buses_taxis" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="things_to_do" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -978,7 +979,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>top_picks</t>
+          <t>things_to_do</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -986,14 +987,14 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Order 18. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+          <t>Order 18. Key: station_slug + name. One row per place under "Things to do". The grey line under the name is kind · location · cost; map_url is the Map button. Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Things to do.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>station_top_picks</t>
+          <t>top_picks</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
@@ -1001,84 +1002,98 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Order 19. location_type: inside/outside/inside_outside.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30"/>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+          <t>Order 19. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>station_top_picks</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Order 20. location_type: inside/outside/inside_outside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>New columns (all optional - delete the column to leave stored values untouched):</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
-        </is>
-      </c>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
+          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
+          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
+          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
+          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
+          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
+          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
+          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
           <t>practical_tips: bullets under 'Practical tips'. faqs: 'FAQ' list; answer is required. Both are also editable in Admin &gt; Stations &gt; Practical tips / FAQs.</t>
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42"/>
     <row r="43"/>
     <row r="44"/>
@@ -2002,26 +2017,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>slug</t>
+          <t>station_slug</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
@@ -2036,110 +2053,118 @@
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>kind</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
+          <t>kind_japanese</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>location_japanese</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>cost_japanese</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>description_japanese</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>entry_fee</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>entry_fee_japanese</t>
-        </is>
-      </c>
-      <c r="I1" s="5" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-      <c r="J1" s="5" t="inlineStr">
-        <is>
-          <t>notes_japanese</t>
-        </is>
-      </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>map_url</t>
         </is>
       </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>#asakura-museum</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>Asakura Museum</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>朝倉彫塑館</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>museum</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>Sculptor's former home</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>彫刻家の旧居</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>500 JPY</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>500円</t>
-        </is>
-      </c>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>Closed Mondays</t>
-        </is>
-      </c>
-      <c r="J2" s="6" t="inlineStr">
-        <is>
-          <t>月曜休館</t>
-        </is>
-      </c>
-      <c r="K2" s="6" t="inlineStr">
-        <is>
-          <t>https://maps.google.com/?q=Asakura+Museum</t>
-        </is>
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>#tokyo</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Imperial Palace East Gardens</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>皇居東御苑</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Garden</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>庭園</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Marunouchi North Exit, about 13 min</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>丸の内北口から徒歩約13分</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>無料</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>Enter by Ote-mon Gate, the one facing Tokyo Station; you take a plastic ticket at the gate and hand it back when you leave. Allow about an hour. Open …</t>
+        </is>
+      </c>
+      <c r="K2" s="7" t="inlineStr"/>
+      <c r="L2" s="7" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Imperial+Palace+East+Gardens</t>
+        </is>
+      </c>
+      <c r="M2" s="7" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"landmark,food,shopping,museum,park,temple"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -2231,6 +2256,153 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>name_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>description_japanese</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>entry_fee</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>entry_fee_japanese</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>notes_japanese</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>map_url</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#asakura-museum</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Asakura Museum</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>朝倉彫塑館</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>museum</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Sculptor's former home</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>彫刻家の旧居</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>500 JPY</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>500円</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>Closed Mondays</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>月曜休館</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>https://maps.google.com/?q=Asakura+Museum</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"landmark,food,shopping,museum,park,temple"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Station page: Hotels (Booking.com link) and Restaurants sections, admin pages, importer, template
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -26,8 +26,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="facility_guide" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="buses_taxis" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="things_to_do" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hotels" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurants" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -625,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -994,7 +996,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>top_picks</t>
+          <t>hotels</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
@@ -1002,14 +1004,14 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Order 19. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+          <t>Order 19. Key: station_slug + name. One row per hotel under "Hotels": kind · location is the grey line; map_url = Map button; booking_url = the "Check prices" button (Booking.com link; leave empty to hide the button). Photos: Admin &gt; Stations &gt; Hotels.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>station_top_picks</t>
+          <t>restaurants</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1017,87 +1019,116 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Order 20. location_type: inside/outside/inside_outside.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31"/>
+          <t>Order 20. Key: station_slug + name. One row per place under "Restaurants": kind · location is the grey line; map_url = Map button. The note above the list is the stations column restaurants_note (**text** = bold). Photos: Admin &gt; Stations &gt; Restaurants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>top_picks</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Order 21. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+        </is>
+      </c>
+    </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>station_top_picks</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Order 22. location_type: inside/outside/inside_outside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>New columns (all optional - delete the column to leave stored values untouched):</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
-        </is>
-      </c>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
+          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
+          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
+          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
+          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
+          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
+          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
           <t>practical_tips: bullets under 'Practical tips'. faqs: 'FAQ' list; answer is required. Both are also editable in Admin &gt; Stations &gt; Practical tips / FAQs.</t>
         </is>
       </c>
     </row>
-    <row r="42"/>
-    <row r="43"/>
     <row r="44"/>
     <row r="45"/>
+    <row r="46"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2261,6 +2292,287 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>name_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>kind_japanese</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>location_japanese</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>description_japanese</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>map_url</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>booking_url</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>#tokyo</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>The Tokyo Station Hotel</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>東京ステーションホテル</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>In the station building</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>駅舎内</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Marunouchi South Exit, directly connected</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>丸の内南口直結</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Hotel inside the red-brick Marunouchi station building; it opened on November 2, 1915, one year after the station.</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr"/>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=The+Tokyo+Station+Hotel</t>
+        </is>
+      </c>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/searchresults.html?ss=The+Tokyo+Station+Hotel</t>
+        </is>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>name_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>kind_japanese</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>location_japanese</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>description_japanese</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>map_url</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>#tokyo</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Rokurinsha</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>六厘舎</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Tsukemen</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>つけ麺</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Tokyo Ramen Street, First Avenue B1 south end</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>東京ラーメンストリート</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>The best-known shop on Tokyo Ramen Street, for tsukemen: thick noodles dipped into a separate bowl of rich broth. Buy a ticket at the machine by the d…</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr"/>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Rokurinsha</t>
+        </is>
+      </c>
+      <c r="K2" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2402,7 +2714,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2624,7 +2936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AD2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2655,6 +2967,8 @@
     <col width="36" customWidth="1" min="26" max="26"/>
     <col width="44" customWidth="1" min="27" max="27"/>
     <col width="36" customWidth="1" min="28" max="28"/>
+    <col width="40" customWidth="1" min="29" max="29"/>
+    <col width="40" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2796,6 +3110,16 @@
       <c r="AB1" s="5" t="inlineStr">
         <is>
           <t>exits_note_japanese</t>
+        </is>
+      </c>
+      <c r="AC1" s="5" t="inlineStr">
+        <is>
+          <t>restaurants_note</t>
+        </is>
+      </c>
+      <c r="AD1" s="5" t="inlineStr">
+        <is>
+          <t>restaurants_note_japanese</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hotels and restaurants as their own admin records assigned to stations (top-pick style), importer and template updated
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -26,10 +26,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="facility_guide" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="buses_taxis" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="things_to_do" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hotels" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurants" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hotels" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurants" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_hotels" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_restaurants" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -627,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -996,7 +998,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>hotels</t>
+          <t>top_picks</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
@@ -1004,14 +1006,14 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Order 19. Key: station_slug + name. One row per hotel under "Hotels": kind · location is the grey line; map_url = Map button; booking_url = the "Check prices" button (Booking.com link; leave empty to hide the button). Photos: Admin &gt; Stations &gt; Hotels.</t>
+          <t>Order 19. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>restaurants</t>
+          <t>station_top_picks</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1019,14 +1021,14 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Order 20. Key: station_slug + name. One row per place under "Restaurants": kind · location is the grey line; map_url = Map button. The note above the list is the stations column restaurants_note (**text** = bold). Photos: Admin &gt; Stations &gt; Restaurants.</t>
+          <t>Order 20. location_type: inside/outside/inside_outside.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>top_picks</t>
+          <t>hotels</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
@@ -1034,14 +1036,14 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Order 21. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+          <t>Order 21. Key: slug. A hotel record (like top_picks): grey line = kind; map_url = Map button; booking_url = the "Check prices" button (Booking.com link; empty hides it). Photos: Admin &gt; Hotels.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>station_top_picks</t>
+          <t>restaurants</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1049,86 +1051,121 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Order 22. location_type: inside/outside/inside_outside.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33"/>
+          <t>Order 22. Key: slug. A restaurant record: grey line = kind; map_url = Map button. The note above the list is the stations column restaurants_note (**text** = bold). Photos: Admin &gt; Restaurants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>station_hotels</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Order 23. Key: station_slug + hotel_slug. Puts a hotel on a station page: location = where it is from that station (grey line, after kind), sort_order = position.</t>
+        </is>
+      </c>
+    </row>
     <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>station_restaurants</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Order 24. Key: station_slug + restaurant_slug. Puts a restaurant on a station page: location = where it is from that station, sort_order = position.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>New columns (all optional - delete the column to leave stored values untouched):</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
-        </is>
-      </c>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
+          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
+          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
+          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
+          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
+          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
+          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
           <t>practical_tips: bullets under 'Practical tips'. faqs: 'FAQ' list; answer is required. Both are also editable in Admin &gt; Stations &gt; Practical tips / FAQs.</t>
         </is>
       </c>
     </row>
-    <row r="44"/>
-    <row r="45"/>
     <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2292,287 +2329,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="70" customWidth="1" min="8" max="8"/>
-    <col width="50" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>station_slug</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>name_japanese</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>kind</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>kind_japanese</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>location</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>location_japanese</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="I1" s="5" t="inlineStr">
-        <is>
-          <t>description_japanese</t>
-        </is>
-      </c>
-      <c r="J1" s="5" t="inlineStr">
-        <is>
-          <t>map_url</t>
-        </is>
-      </c>
-      <c r="K1" s="5" t="inlineStr">
-        <is>
-          <t>booking_url</t>
-        </is>
-      </c>
-      <c r="L1" s="5" t="inlineStr">
-        <is>
-          <t>sort_order</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>#tokyo</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>The Tokyo Station Hotel</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>東京ステーションホテル</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>In the station building</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>駅舎内</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>Marunouchi South Exit, directly connected</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
-        <is>
-          <t>丸の内南口直結</t>
-        </is>
-      </c>
-      <c r="H2" s="7" t="inlineStr">
-        <is>
-          <t>Hotel inside the red-brick Marunouchi station building; it opened on November 2, 1915, one year after the station.</t>
-        </is>
-      </c>
-      <c r="I2" s="7" t="inlineStr"/>
-      <c r="J2" s="7" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=The+Tokyo+Station+Hotel</t>
-        </is>
-      </c>
-      <c r="K2" s="7" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/searchresults.html?ss=The+Tokyo+Station+Hotel</t>
-        </is>
-      </c>
-      <c r="L2" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="70" customWidth="1" min="8" max="8"/>
-    <col width="50" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>station_slug</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>name_japanese</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>kind</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>kind_japanese</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>location</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>location_japanese</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="I1" s="5" t="inlineStr">
-        <is>
-          <t>description_japanese</t>
-        </is>
-      </c>
-      <c r="J1" s="5" t="inlineStr">
-        <is>
-          <t>map_url</t>
-        </is>
-      </c>
-      <c r="K1" s="5" t="inlineStr">
-        <is>
-          <t>sort_order</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>#tokyo</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>Rokurinsha</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>六厘舎</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>Tsukemen</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>つけ麺</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>Tokyo Ramen Street, First Avenue B1 south end</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
-        <is>
-          <t>東京ラーメンストリート</t>
-        </is>
-      </c>
-      <c r="H2" s="7" t="inlineStr">
-        <is>
-          <t>The best-known shop on Tokyo Ramen Street, for tsukemen: thick noodles dipped into a separate bowl of rich broth. Buy a ticket at the machine by the d…</t>
-        </is>
-      </c>
-      <c r="I2" s="7" t="inlineStr"/>
-      <c r="J2" s="7" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Rokurinsha</t>
-        </is>
-      </c>
-      <c r="K2" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2714,7 +2470,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2788,6 +2544,376 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>name_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>kind_japanese</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>description_japanese</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>map_url</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>booking_url</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>#the-tokyo-station-hotel</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>The Tokyo Station Hotel</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>東京ステーションホテル</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>In the station building</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>駅舎内</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Hotel inside the red-brick Marunouchi station building; it opened on November 2, 1915, one year after the station.</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr"/>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=The+Tokyo+Station+Hotel</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/searchresults.html?ss=The+Tokyo+Station+Hotel</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>name_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>kind_japanese</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>description_japanese</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>map_url</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>#rokurinsha</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Rokurinsha</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>六厘舎</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Tsukemen</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>つけ麺</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>The best-known shop on Tokyo Ramen Street, for tsukemen: thick noodles dipped into a separate bowl of rich broth. Buy a ticket at the machine by the d…</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr"/>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Rokurinsha</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>hotel_slug</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>location_japanese</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>#tokyo</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>the-tokyo-station-hotel</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Marunouchi South Exit, directly connected</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>丸の内南口直結</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>restaurant_slug</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>location_japanese</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>#tokyo</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>rokurinsha</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Tokyo Ramen Street, First Avenue B1 south end · Yaesu South Exit side</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr"/>
+      <c r="E2" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Which exit?: side tabs, exit chips, place filter, operator map link; admin sides<->exits and places; importer sheet exit_places and sides.exits
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -17,21 +17,22 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exits" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="platforms" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sides" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="routes" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tips" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="seasons" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="practical_tips" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="faqs" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="day_trips" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="facility_guide" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="buses_taxis" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="things_to_do" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hotels" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurants" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_hotels" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_restaurants" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exit_places" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="routes" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tips" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="seasons" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="practical_tips" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="faqs" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="day_trips" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="facility_guide" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="buses_taxis" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="things_to_do" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hotels" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurants" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_hotels" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_restaurants" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -629,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -863,309 +864,355 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>routes</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>10</v>
+          <t>exit_places</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Order 10. Key: station_slug + from_place + route. One row per way of getting to the station ("Getting there" table). The footnote is the stations column routes_note.</t>
+          <t>Order 10. Key: station_slug + name. "Which exit?" on the public page: one row per place (sights / food / hotels / transport / help). category: sights, food, hotels, transport or help. exits = the exits that lead to it, "Exit name=short note" separated by | (exit names must exist in exits); exit_notes_japanese = "Exit name=日本語メモ". Do not use = or | inside a note.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>tips</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>11</v>
+          <t>routes</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Order 11. Key: station_slug + tip. One row per bullet under "Exits &amp; station tips". Exit photos are uploaded in Admin &gt; Manage Exits; the table above them comes from the exits sheet (name + description).</t>
+          <t>Order 11. Key: station_slug + from_place + route. One row per way of getting to the station ("Getting there" table). The footnote is the stations column routes_note.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>seasons</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>12</v>
+          <t>tips</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Order 12. Key: station_slug + season. season: spring/summer/autumn/winter (one row each). One row per season of "When to visit": months (red label, e.g. Mar – May) + description.</t>
+          <t>Order 12. Key: station_slug + tip. One row per bullet under "Exits &amp; station tips". Exit photos are uploaded in Admin &gt; Manage Exits; the table above them comes from the exits sheet (name + description).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>practical_tips</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="n">
-        <v>13</v>
+          <t>seasons</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Order 13. Key: station_slug + tip. One row per bullet under "Practical tips".</t>
+          <t>Order 13. Key: station_slug + season. season: spring/summer/autumn/winter (one row each). One row per season of "When to visit": months (red label, e.g. Mar – May) + description.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>faqs</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>14</v>
+          <t>practical_tips</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Order 14. Key: station_slug + question. One row per FAQ (question + answer, opens when clicked).</t>
+          <t>Order 14. Key: station_slug + tip. One row per bullet under "Practical tips".</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>day_trips</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>15</v>
+          <t>faqs</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Order 15. Key: station_slug + name. One row per place under "Day trips": travel_time (e.g. ≈ 25–40 min) · transport (e.g. JR lines, direct), description, map_url (the Map button). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Day trips.</t>
+          <t>Order 15. Key: station_slug + question. One row per FAQ (question + answer, opens when clicked).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>facility_guide</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>16</v>
+          <t>day_trips</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Order 16. Key: station_slug + name. The public "Facilities" section (not the facility icons of the floor map): a row with a description is listed in the table (Facility / Where and what to know); a row with a photo also gets a photo card (name + photo_caption). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Facilities guide.</t>
+          <t>Order 16. Key: station_slug + name. One row per place under "Day trips": travel_time (e.g. ≈ 25–40 min) · transport (e.g. JR lines, direct), description, map_url (the Map button). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Day trips.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>buses_taxis</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>17</v>
+          <t>facility_guide</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Order 17. Key: station_slug + place. The public "Buses &amp; taxis" section: a row with service or notes is listed in the table (Where / Service / Notes); a row with a photo also gets a photo card (photo_title, or place, + photo_caption). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Buses &amp; taxis.</t>
+          <t>Order 17. Key: station_slug + name. The public "Facilities" section (not the facility icons of the floor map): a row with a description is listed in the table (Facility / Where and what to know); a row with a photo also gets a photo card (name + photo_caption). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Facilities guide.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>things_to_do</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="n">
-        <v>18</v>
+          <t>buses_taxis</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Order 18. Key: station_slug + name. One row per place under "Things to do". The grey line under the name is kind · location · cost; map_url is the Map button. Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Things to do.</t>
+          <t>Order 18. Key: station_slug + place. The public "Buses &amp; taxis" section: a row with service or notes is listed in the table (Where / Service / Notes); a row with a photo also gets a photo card (photo_title, or place, + photo_caption). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Buses &amp; taxis.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>top_picks</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="n">
-        <v>19</v>
+          <t>things_to_do</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Order 19. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+          <t>Order 19. Key: station_slug + name. One row per place under "Things to do". The grey line under the name is kind · location · cost; map_url is the Map button. Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Things to do.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>station_top_picks</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="n">
-        <v>20</v>
+          <t>top_picks</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Order 20. location_type: inside/outside/inside_outside.</t>
+          <t>Order 20. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>hotels</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="n">
-        <v>21</v>
+          <t>station_top_picks</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Order 21. Key: slug. A hotel record (like top_picks): grey line = kind; map_url = Map button; booking_url = the "Check prices" button (Booking.com link; empty hides it). Photos: Admin &gt; Hotels.</t>
+          <t>Order 21. location_type: inside/outside/inside_outside.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>restaurants</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="n">
-        <v>22</v>
+          <t>hotels</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Order 22. Key: slug. A restaurant record: grey line = kind; map_url = Map button. The note above the list is the stations column restaurants_note (**text** = bold). Photos: Admin &gt; Restaurants.</t>
+          <t>Order 22. Key: slug. A hotel record (like top_picks): grey line = kind; map_url = Map button; booking_url = the "Check prices" button (Booking.com link; empty hides it). Photos: Admin &gt; Hotels.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>station_hotels</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="n">
-        <v>23</v>
+          <t>restaurants</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Order 23. Key: station_slug + hotel_slug. Puts a hotel on a station page: location = where it is from that station (grey line, after kind), sort_order = position.</t>
+          <t>Order 23. Key: slug. A restaurant record: grey line = kind; map_url = Map button. The note above the list is the stations column restaurants_note (**text** = bold). Photos: Admin &gt; Restaurants.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
+          <t>station_hotels</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Order 24. Key: station_slug + hotel_slug. Puts a hotel on a station page: location = where it is from that station (grey line, after kind), sort_order = position.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
           <t>station_restaurants</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Order 24. Key: station_slug + restaurant_slug. Puts a restaurant on a station page: location = where it is from that station, sort_order = position.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35"/>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Order 25. Key: station_slug + restaurant_slug. Puts a restaurant on a station page: location = where it is from that station, sort_order = position.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>New columns (all optional - delete the column to leave stored values untouched):</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
-        </is>
-      </c>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
+          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
+          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
+          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
+          <t>sides: 'exits' = exit names of this side, separated by | (they appear as tabs/chips in "Which exit?"; a side with no exits lists all). exit_places: the places in "Which exit?" - see its row above. The "Full station map" button uses the operator's website_url from the operators sheet.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
+          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
+          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
+          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
           <t>practical_tips: bullets under 'Practical tips'. faqs: 'FAQ' list; answer is required. Both are also editable in Admin &gt; Stations &gt; Practical tips / FAQs.</t>
         </is>
       </c>
     </row>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1177,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1188,6 +1235,7 @@
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1231,6 +1279,11 @@
           <t>sort_order</t>
         </is>
       </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>exits</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -1270,6 +1323,11 @@
       </c>
       <c r="H2" s="6" t="n">
         <v>1</v>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>Marunouchi North Exit|Marunouchi Central Exit|Marunouchi South Exit</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1278,6 +1336,101 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>name_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>exits</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>exit_notes_japanese</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>#tokyo</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>KITTE &amp; KITTE Garden</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>KITTE・KITTEガーデン</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>sights</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Marunouchi South Exit=1 min|Marunouchi Underground North Exit=underground</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Marunouchi South Exit=徒歩1分|Marunouchi Underground North Exit=地下直結</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1405,7 +1558,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1467,7 +1620,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1553,7 +1706,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1620,7 +1773,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1707,7 +1860,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1846,7 +1999,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1945,7 +2098,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2079,7 +2232,94 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>name_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>description_japanese</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>website_url</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#jr-east</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>JR East</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>JR東日本</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Main railway operator in Kanto</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>関東の主要鉄道会社</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>https://www.jreast.co.jp</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2236,94 +2476,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>slug</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>name_japanese</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>description_japanese</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>website_url</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>#jr-east</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>JR East</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>JR東日本</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>Main railway operator in Kanto</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>関東の主要鉄道会社</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>https://www.jreast.co.jp</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2470,7 +2623,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2547,7 +2700,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2662,7 +2815,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2767,7 +2920,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2844,7 +2997,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
One table per place type: sights/food/hotels with exit + walking minutes
Things to do, Which exit? and map Top picks now read the same records
(top_picks, restaurants, hotels + station links with exit and minutes).
Migration 0045 moves station_things and sights/food/hotels exit places over.
Importer: things_to_do sheet removed; exit_name/walking_minutes/location columns;
template updated for all three merges.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -21,18 +21,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="routes" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tips" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="seasons" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="practical_tips" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="faqs" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="day_trips" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="facility_guide" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="buses_taxis" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="things_to_do" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hotels" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurants" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_hotels" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_restaurants" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="faqs" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="day_trips" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="buses_taxis" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hotels" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurants" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_hotels" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_restaurants" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -812,7 +809,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Order 6. floor_name must exist in floors for that station. exits = nearby exits of this facility, exit names from the exits sheet separated by ; (empty cell clears them). note is a separate column. location_type: inside/outside. facility_slug must already exist in Admin &gt; Facilities (the importer never creates or changes facilities).</t>
+          <t>Order 6. Key: station_slug + floor_name + facility_slug. ONE facilities table (used by the map popup and the station page): floor, exits (exit names separated by ;), location_type inside/outside, icon (from the facility), description (+ _japanese) and optional photo_caption. facility_slug must already exist in Admin &gt; Facilities. Photos: Admin &gt; Stations &gt; Facilities.</t>
         </is>
       </c>
     </row>
@@ -874,7 +871,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Order 10. Key: station_slug + name. "Which exit?" on the public page: one row per place (sights / food / hotels / transport / help). category: sights, food, hotels, transport or help. exits = the exits that lead to it, "Exit name=short note" separated by | (exit names must exist in exits); exit_notes_japanese = "Exit name=日本語メモ". Do not use = or | inside a note.</t>
+          <t>Order 10. Key: station_slug + name. "Which exit?": only category transport or help here. Sights, food and hotels appear there automatically from station_top_picks / station_restaurants / station_hotels (rows with an exit_name). exits = "Exit name=short note" separated by |; exit_notes_japanese = "Exit name=日本語メモ".</t>
         </is>
       </c>
     </row>
@@ -908,7 +905,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Order 12. Key: station_slug + tip. One row per bullet under "Exits &amp; station tips". Exit photos are uploaded in Admin &gt; Manage Exits; the table above them comes from the exits sheet (name + description).</t>
+          <t>Order 12. Key: station_slug + section + tip. section = exits (bullets under "Exits &amp; station tips") or practical (bullets under "Practical tips"); empty = exits.</t>
         </is>
       </c>
     </row>
@@ -932,212 +929,190 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>practical_tips</t>
+          <t>faqs</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Order 14. Key: station_slug + tip. One row per bullet under "Practical tips".</t>
+          <t>Order 15. Key: station_slug + question. One row per FAQ (question + answer, opens when clicked).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>faqs</t>
+          <t>day_trips</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Order 15. Key: station_slug + question. One row per FAQ (question + answer, opens when clicked).</t>
+          <t>Order 16. Key: station_slug + name. One row per place under "Day trips": travel_time (e.g. ≈ 25–40 min) · transport (e.g. JR lines, direct), description, map_url (the Map button). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Day trips.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>day_trips</t>
+          <t>buses_taxis</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Order 16. Key: station_slug + name. One row per place under "Day trips": travel_time (e.g. ≈ 25–40 min) · transport (e.g. JR lines, direct), description, map_url (the Map button). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Day trips.</t>
+          <t>Order 18. Key: station_slug + place. The public "Buses &amp; taxis" section: a row with service or notes is listed in the table (Where / Service / Notes); a row with a photo also gets a photo card (photo_title, or place, + photo_caption). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Buses &amp; taxis.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>facility_guide</t>
+          <t>top_picks</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Order 17. Key: station_slug + name. The public "Facilities" section (not the facility icons of the floor map): a row with a description is listed in the table (Facility / Where and what to know); a row with a photo also gets a photo card (name + photo_caption). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Facilities guide.</t>
+          <t>Order 20. Key: slug. One sights table: used by Things to do, Which exit? and the map's Top picks. kind = grey line (e.g. Garden), category: landmark/food/shopping/museum/park/temple, entry_fee = cost. Photos: Admin &gt; Top picks.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>buses_taxis</t>
+          <t>station_top_picks</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Order 18. Key: station_slug + place. The public "Buses &amp; taxis" section: a row with service or notes is listed in the table (Where / Service / Notes); a row with a photo also gets a photo card (photo_title, or place, + photo_caption). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Buses &amp; taxis.</t>
+          <t>Order 21. Key: station_slug + top_pick_slug. Puts a sight on a station: exit_name (from exits sheet), walking_minutes, location_type inside/outside/inside_outside, location (+ _japanese) free text, sort_order.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>things_to_do</t>
+          <t>hotels</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Order 19. Key: station_slug + name. One row per place under "Things to do". The grey line under the name is kind · location · cost; map_url is the Map button. Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Things to do.</t>
+          <t>Order 22. Key: slug. A hotel record (like top_picks): grey line = kind; map_url = Map button; booking_url = the "Check prices" button (Booking.com link; empty hides it). Photos: Admin &gt; Hotels.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>top_picks</t>
+          <t>restaurants</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Order 20. category: landmark/food/shopping/museum/park/temple. Photos cannot be uploaded in Excel; add them in Admin &gt; Top picks.</t>
+          <t>Order 23. Key: slug. A restaurant record: grey line = kind; map_url = Map button. The note above the list is the stations column restaurants_note (**text** = bold). Photos: Admin &gt; Restaurants.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>station_top_picks</t>
+          <t>station_hotels</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Order 21. location_type: inside/outside/inside_outside.</t>
+          <t>Order 24. Key: station_slug + hotel_slug. exit_name (from exits sheet), walking_minutes, location (free text), sort_order. Shown in Hotels and in Which exit?.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>hotels</t>
+          <t>station_restaurants</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>25</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Order 22. Key: slug. A hotel record (like top_picks): grey line = kind; map_url = Map button; booking_url = the "Check prices" button (Booking.com link; empty hides it). Photos: Admin &gt; Hotels.</t>
+          <t>Order 25. Key: station_slug + restaurant_slug. exit_name (from exits sheet), walking_minutes, location (free text), sort_order. Shown in Restaurants and in Which exit?.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>restaurants</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Order 23. Key: slug. A restaurant record: grey line = kind; map_url = Map button. The note above the list is the stations column restaurants_note (**text** = bold). Photos: Admin &gt; Restaurants.</t>
-        </is>
-      </c>
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>station_hotels</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Order 24. Key: station_slug + hotel_slug. Puts a hotel on a station page: location = where it is from that station (grey line, after kind), sort_order = position.</t>
-        </is>
-      </c>
+          <t>New columns (all optional - delete the column to leave stored values untouched):</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>station_restaurants</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Order 25. Key: station_slug + restaurant_slug. Puts a restaurant on a station page: location = where it is from that station, sort_order = position.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36"/>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
+        </is>
+      </c>
+    </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>New columns (all optional - delete the column to leave stored values untouched):</t>
+          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
         </is>
       </c>
       <c r="B37" s="2" t="n"/>
@@ -1146,72 +1121,56 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
+          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
+          <t>sides: 'exits' = exit names of this side, separated by | (they appear as tabs/chips in "Which exit?"; a side with no exits lists all). exit_places: the places in "Which exit?" - see its row above. The "Full station map" button uses the operator's website_url from the operators sheet.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
+          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
+          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>sides: 'exits' = exit names of this side, separated by | (they appear as tabs/chips in "Which exit?"; a side with no exits lists all). exit_places: the places in "Which exit?" - see its row above. The "Full station map" button uses the operator's website_url from the operators sheet.</t>
+          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
+          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
-        </is>
-      </c>
+      <c r="A44" s="2" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
-        </is>
-      </c>
+      <c r="A45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
-        </is>
-      </c>
+      <c r="A46" s="2" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>practical_tips: bullets under 'Practical tips'. faqs: 'FAQ' list; answer is required. Both are also editable in Admin &gt; Stations &gt; Practical tips / FAQs.</t>
-        </is>
-      </c>
+      <c r="A47" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1564,13 +1523,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1581,15 +1541,20 @@
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
           <t>tip</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>tip_japanese</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>sort_order</t>
         </is>
@@ -1598,20 +1563,25 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>#tokyo</t>
+          <t>#example-station</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>The Marunouchi Central gate is IC card only and open 9:30-17:00; use the North or South gates with a paper ticket.</t>
+          <t>exits</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>丸の内中央口はIC専用（9:30〜17:00）。紙のきっぷは北口・南口へ。</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="n">
+          <t>One bullet of text</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>箇条書きの文</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1712,73 +1682,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>station_slug</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>tip</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>tip_japanese</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>sort_order</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>#tokyo</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>The Tokaido-Sanyo Shinkansen (JR Central) uses platforms 14–19 and blue gates; the Tohoku, Joetsu and Hokuriku Shinkansen (JR East) use platforms 20–23 and green gates. Check which colour your train belongs to before you follow the signs.</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>東海道・山陽新幹線は14〜19番線（青い改札）、東北・上越・北陸新幹線は20〜23番線（緑の改札）です。</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1860,7 +1763,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1999,106 +1902,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="80" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>station_slug</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>name_japanese</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>description_japanese</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>photo_caption</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>photo_caption_japanese</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>sort_order</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>#tokyo</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>Coin lockers</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>コインロッカー</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>The locker banks we checked near the Marunouchi gates on 8 October 2026 cost ¥500 (S), ¥700 (M) and ¥900 (L). All are 34 cm wide and 65 cm deep; the height is 33 cm (S), 50 cm (M) or 86 cm (L). The ma…</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr"/>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>From ¥500. This bank takes IC card, credit card or QR payment, not cash.</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr"/>
-      <c r="H2" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2232,6 +2036,253 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>name_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>kind_japanese</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>description_japanese</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>entry_fee</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>entry_fee_japanese</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>notes_japanese</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>map_url</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#example-sight</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Example Garden</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>例の庭園</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Garden</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>庭園</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>park</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="6" t="n"/>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="6" t="n"/>
+      <c r="L2" s="6" t="n"/>
+      <c r="M2" s="6" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"landmark,food,shopping,museum,park,temple"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>top_pick_slug</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>exit_name</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>walking_minutes</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>location_type</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>location_japanese</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#example-station</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>example-sight</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>outside</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="n"/>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"inside,outside,inside_outside"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2320,387 +2371,6 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="70" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>station_slug</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>name_japanese</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>kind</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>kind_japanese</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>location</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>location_japanese</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>cost</t>
-        </is>
-      </c>
-      <c r="I1" s="5" t="inlineStr">
-        <is>
-          <t>cost_japanese</t>
-        </is>
-      </c>
-      <c r="J1" s="5" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="K1" s="5" t="inlineStr">
-        <is>
-          <t>description_japanese</t>
-        </is>
-      </c>
-      <c r="L1" s="5" t="inlineStr">
-        <is>
-          <t>map_url</t>
-        </is>
-      </c>
-      <c r="M1" s="5" t="inlineStr">
-        <is>
-          <t>sort_order</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>#tokyo</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>Imperial Palace East Gardens</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>皇居東御苑</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>Garden</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>庭園</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>Marunouchi North Exit, about 13 min</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
-        <is>
-          <t>丸の内北口から徒歩約13分</t>
-        </is>
-      </c>
-      <c r="H2" s="7" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="I2" s="7" t="inlineStr">
-        <is>
-          <t>無料</t>
-        </is>
-      </c>
-      <c r="J2" s="7" t="inlineStr">
-        <is>
-          <t>Enter by Ote-mon Gate, the one facing Tokyo Station; you take a plastic ticket at the gate and hand it back when you leave. Allow about an hour. Open …</t>
-        </is>
-      </c>
-      <c r="K2" s="7" t="inlineStr"/>
-      <c r="L2" s="7" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Imperial+Palace+East+Gardens</t>
-        </is>
-      </c>
-      <c r="M2" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>slug</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>name_japanese</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>description_japanese</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>entry_fee</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>entry_fee_japanese</t>
-        </is>
-      </c>
-      <c r="I1" s="5" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-      <c r="J1" s="5" t="inlineStr">
-        <is>
-          <t>notes_japanese</t>
-        </is>
-      </c>
-      <c r="K1" s="5" t="inlineStr">
-        <is>
-          <t>map_url</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>#asakura-museum</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>Asakura Museum</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>朝倉彫塑館</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>museum</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>Sculptor's former home</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>彫刻家の旧居</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>500 JPY</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>500円</t>
-        </is>
-      </c>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>Closed Mondays</t>
-        </is>
-      </c>
-      <c r="J2" s="6" t="inlineStr">
-        <is>
-          <t>月曜休館</t>
-        </is>
-      </c>
-      <c r="K2" s="6" t="inlineStr">
-        <is>
-          <t>https://maps.google.com/?q=Asakura+Museum</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"landmark,food,shopping,museum,park,temple"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>station_slug</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>top_pick_slug</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>walking_minutes</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>location_type</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>sort_order</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>#nishi-nippori</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>asakura-museum</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>outside</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"inside,outside,inside_outside"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2815,7 +2485,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2920,22 +2590,22 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
@@ -2953,15 +2623,25 @@
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
+          <t>exit_name</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>walking_minutes</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
           <t>location</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>location_japanese</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>sort_order</t>
         </is>
@@ -2970,25 +2650,25 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>#tokyo</t>
+          <t>#example-station</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>the-tokyo-station-hotel</t>
+          <t>example-hotel</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Marunouchi South Exit, directly connected</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>丸の内南口直結</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="n">
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" s="7" t="n"/>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2997,22 +2677,22 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
@@ -3030,15 +2710,25 @@
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
+          <t>exit_name</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>walking_minutes</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
           <t>location</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>location_japanese</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>sort_order</t>
         </is>
@@ -3047,21 +2737,25 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>#tokyo</t>
+          <t>#example-station</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>rokurinsha</t>
+          <t>example-restaurant</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Tokyo Ramen Street, First Avenue B1 south end · Yaesu South Exit side</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr"/>
-      <c r="E2" s="7" t="n">
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="7" t="n"/>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3687,7 +3381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3695,9 +3389,12 @@
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3723,25 +3420,35 @@
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
+          <t>location_type</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
           <t>facility_count</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
-          <t>note_japanese</t>
+          <t>description</t>
         </is>
       </c>
       <c r="H1" s="5" t="inlineStr">
         <is>
-          <t>location_type</t>
+          <t>description_japanese</t>
         </is>
       </c>
       <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>photo_caption</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>photo_caption_japanese</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>sort_order</t>
         </is>
@@ -3750,7 +3457,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>#nishi-nippori</t>
+          <t>#example-station</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
@@ -3760,33 +3467,35 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>elevator</t>
+          <t>toilet</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>North Exit; South Exit</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="n">
+          <t>A1;A2</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>inside</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>Near the north gate</t>
-        </is>
-      </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>北改札の近く</t>
+          <t>Where it is and what to know</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>inside</t>
-        </is>
-      </c>
-      <c r="I2" s="6" t="n">
+          <t>場所と注意点</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="6" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Facilities: separate texts for map popup, station page table and photo caption (migration 0047); admin groups them with where-it-shows labels; importer popup_note + description
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -809,7 +809,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Order 6. Key: station_slug + floor_name + facility_slug. ONE facilities table (used by the map popup and the station page): floor, exits (exit names separated by ;), location_type inside/outside/inside_outside, icon (from the facility), description (+ _japanese) and optional photo_caption. facility_slug must already exist in Admin &gt; Facilities. Photos: Admin &gt; Stations &gt; Facilities.</t>
+          <t>Key: station_slug + floor_name + facility_slug. ONE facilities table with three separate texts: popup_note (+ _japanese) = the short text of the MAP POPUP; description (+ _japanese) = the "Facilities" TABLE on the station page (empty = not listed there); photo_caption (+ _japanese) = the caption of the PHOTO card. Also: exits (exit names separated by ;), location_type inside/outside/inside_outside, facility_count. facility_slug must exist in Admin &gt; Facilities. Photos: Admin &gt; Stations &gt; Facilities.</t>
         </is>
       </c>
     </row>
@@ -3381,20 +3381,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3430,25 +3432,35 @@
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
+          <t>popup_note</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>popup_note_japanese</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>description_japanese</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>photo_caption</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>photo_caption_japanese</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>sort_order</t>
         </is>
@@ -3485,17 +3497,27 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>Where it is and what to know</t>
+          <t>Short text for the map popup</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>場所と注意点</t>
-        </is>
-      </c>
-      <c r="I2" s="6" t="n"/>
-      <c r="J2" s="6" t="n"/>
-      <c r="K2" s="6" t="n">
+          <t>マップ用の短い説明</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>Where it is and what to know (station page table)</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>場所と注意点（駅ページの表）</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="n"/>
+      <c r="L2" s="6" t="n"/>
+      <c r="M2" s="6" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Separate Top picks (main page/map popup) and Things to do (station page): both pick from Places
Adds station_things table (0048), admin sub menu, public page query and importer sheet.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -26,10 +26,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="buses_taxis" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hotels" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurants" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_hotels" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_restaurants" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_things" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hotels" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurants" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_hotels" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_restaurants" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -87,7 +88,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -95,11 +96,12 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -112,6 +114,11 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -204,6 +211,21 @@
 </file>
 
 <file path=xl/comments/comment10.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Template</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Order 11. location_type: inside/outside/inside_outside.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment11.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Template</author>
@@ -627,7 +649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -871,7 +893,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Order 10. Key: station_slug + name. "Which exit?": only category transport or help here. Sights, food and hotels appear there automatically from station_top_picks / station_restaurants / station_hotels (rows with an exit_name). exits = "Exit name=short note" separated by |; exit_notes_japanese = "Exit name=日本語メモ".</t>
+          <t>Order 10. Key: station_slug + name. "Which exit?": only category transport or help here. Sights, food and hotels appear there automatically from station_things / station_restaurants / station_hotels (rows with an exit_name). exits = "Exit name=short note" separated by |; exit_notes_japanese = "Exit name=日本語メモ".</t>
         </is>
       </c>
     </row>
@@ -990,7 +1012,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Order 20. Key: slug. One sights table: used by Things to do, Which exit? and the map's Top picks. kind = grey line (e.g. Garden), category: landmark/food/shopping/museum/park/temple, entry_fee = cost. Photos: Admin &gt; Top picks.</t>
+          <t>Order 20. Key: slug. The PLACES catalog (Admin &gt; Places): one record per place, used by both lists below. kind = grey line (e.g. Garden), category: landmark/food/shopping/museum/park/temple, entry_fee = cost. Photos: Admin &gt; Places.</t>
         </is>
       </c>
     </row>
@@ -1007,96 +1029,102 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Order 21. Key: station_slug + top_pick_slug. Puts a sight on a station: exit_name (from exits sheet), walking_minutes, location_type inside/outside/inside_outside, location (+ _japanese) free text, sort_order.</t>
+          <t>Order 21. Key: station_slug + top_pick_slug. TOP PICKS = the website main page / map popup. Picks a place for a station: exit_name (from exits sheet), walking_minutes, location_type inside/outside/inside_outside, location (+ _japanese) free text, sort_order.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>hotels</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
+          <t>station_things</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>21</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Order 22. Key: slug. A hotel record (like top_picks): grey line = kind; map_url = Map button; booking_url = the "Check prices" button (Booking.com link; empty hides it). Photos: Admin &gt; Hotels.</t>
+          <t>Order 21. Key: station_slug + top_pick_slug. THINGS TO DO = the station page (and "Which exit?"). A separate list from station_top_picks: picks a place from top_picks for this station: exit_name, walking_minutes, location (+ _japanese) free text, sort_order.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>restaurants</t>
+          <t>hotels</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Order 23. Key: slug. A restaurant record: grey line = kind; map_url = Map button. The note above the list is the stations column restaurants_note (**text** = bold). Photos: Admin &gt; Restaurants.</t>
+          <t>Order 22. Key: slug. A hotel record (like top_picks): grey line = kind; map_url = Map button; booking_url = the "Check prices" button (Booking.com link; empty hides it). Photos: Admin &gt; Hotels.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>station_hotels</t>
+          <t>restaurants</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Order 24. Key: station_slug + hotel_slug. exit_name (from exits sheet), walking_minutes, location (free text), sort_order. Shown in Hotels and in Which exit?.</t>
+          <t>Order 23. Key: slug. A restaurant record: grey line = kind; map_url = Map button. The note above the list is the stations column restaurants_note (**text** = bold). Photos: Admin &gt; Restaurants.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
+          <t>station_hotels</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Order 24. Key: station_slug + hotel_slug. exit_name (from exits sheet), walking_minutes, location (free text), sort_order. Shown in Hotels and in Which exit?.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
           <t>station_restaurants</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>Order 25. Key: station_slug + restaurant_slug. exit_name (from exits sheet), walking_minutes, location (free text), sort_order. Shown in Restaurants and in Which exit?.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
-    </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>New columns (all optional - delete the column to leave stored values untouched):</t>
-        </is>
-      </c>
+      <c r="A34" s="2" t="n"/>
       <c r="B34" s="2" t="n"/>
       <c r="C34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
+          <t>New columns (all optional - delete the column to leave stored values untouched):</t>
         </is>
       </c>
       <c r="B35" s="2" t="n"/>
@@ -1105,14 +1133,14 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
+          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
         </is>
       </c>
       <c r="B37" s="2" t="n"/>
@@ -1121,47 +1149,51 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
+          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>sides: 'exits' = exit names of this side, separated by | (they appear as tabs/chips in "Which exit?"; a side with no exits lists all). exit_places: the places in "Which exit?" - see its row above. The "Full station map" button uses the operator's website_url from the operators sheet.</t>
+          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
+          <t>sides: 'exits' = exit names of this side, separated by | (they appear as tabs/chips in "Which exit?"; a side with no exits lists all). exit_places: the places in "Which exit?" - see its row above. The "Full station map" button uses the operator's website_url from the operators sheet.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
+          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
+          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
+          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
           <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
         </is>
       </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n"/>
@@ -1171,6 +1203,9 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2379,6 +2414,97 @@
   <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>top_pick_slug</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>exit_name</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>walking_minutes</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>location_japanese</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+      <c r="H1" s="8" t="n"/>
+      <c r="I1" s="9" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#example-station</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>example-sight</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="6" t="n"/>
+      <c r="G2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="10" t="n"/>
+      <c r="I2" s="9" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
@@ -2485,7 +2611,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2590,7 +2716,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2677,7 +2803,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3381,7 +3507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>

</xml_diff>

<commit_message>
Station places: one table (station_places) with Top pick / Thing to do / Which exit? / Day trip flags
Migration 0049 merges station_top_picks, station_things, station_day_trips and transport/help exit places.
One Places sub menu with a flag form, public page + map popup read the flags, importer sheet station_places.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -17,20 +17,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exits" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="platforms" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sides" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exit_places" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="routes" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tips" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="seasons" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="faqs" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="day_trips" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="buses_taxis" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_top_picks" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_things" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hotels" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurants" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_hotels" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_restaurants" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="routes" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tips" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="seasons" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="faqs" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="buses_taxis" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top_picks" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_places" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hotels" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurants" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_hotels" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="station_restaurants" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -211,21 +208,6 @@
 </file>
 
 <file path=xl/comments/comment10.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Template</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Order 11. location_type: inside/outside/inside_outside.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment11.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Template</author>
@@ -831,7 +813,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Key: station_slug + floor_name + facility_slug. ONE facilities table with three separate texts: popup_note (+ _japanese) = the short text of the MAP POPUP; description (+ _japanese) = the "Facilities" TABLE on the station page (empty = not listed there); photo_caption (+ _japanese) = the caption of the PHOTO card. Also: exits (exit names separated by ;), location_type inside/outside/inside_outside, facility_count. facility_slug must exist in Admin &gt; Facilities. Photos: Admin &gt; Stations &gt; Facilities.</t>
+          <t>Order 6. Key: station_slug + floor_name + facility_slug. ONE facilities table with three separate texts: popup_note (+ _japanese) = the short text of the MAP POPUP; description (+ _japanese) = the "Facilities" TABLE on the station page (empty = not listed there); photo_caption (+ _japanese) = the caption of the PHOTO card. Also: exits (exit names separated by ;), location_type inside/outside/inside_outside, facility_count. facility_slug must exist in Admin &gt; Facilities. Photos: Admin &gt; Stations &gt; Facilities.</t>
         </is>
       </c>
     </row>
@@ -883,248 +865,204 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>exit_places</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+          <t>routes</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>10</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Order 10. Key: station_slug + name. "Which exit?": only category transport or help here. Sights, food and hotels appear there automatically from station_things / station_restaurants / station_hotels (rows with an exit_name). exits = "Exit name=short note" separated by |; exit_notes_japanese = "Exit name=日本語メモ".</t>
+          <t>Order 10. Key: station_slug + from_place + route. One row per way of getting to the station ("Getting there" table). The footnote is the stations column routes_note.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>routes</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+          <t>tips</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>11</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Order 11. Key: station_slug + from_place + route. One row per way of getting to the station ("Getting there" table). The footnote is the stations column routes_note.</t>
+          <t>Order 11. Key: station_slug + section + tip. section = exits (bullets under "Exits &amp; station tips") or practical (bullets under "Practical tips"); empty = exits.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>tips</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+          <t>seasons</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>12</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Order 12. Key: station_slug + section + tip. section = exits (bullets under "Exits &amp; station tips") or practical (bullets under "Practical tips"); empty = exits.</t>
+          <t>Order 12. Key: station_slug + season. season: spring/summer/autumn/winter (one row each). One row per season of "When to visit": months (red label, e.g. Mar – May) + description.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>seasons</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
+          <t>faqs</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>13</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Order 13. Key: station_slug + season. season: spring/summer/autumn/winter (one row each). One row per season of "When to visit": months (red label, e.g. Mar – May) + description.</t>
+          <t>Order 13. Key: station_slug + question. One row per FAQ (question + answer, opens when clicked).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>faqs</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+          <t>buses_taxis</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>14</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Order 15. Key: station_slug + question. One row per FAQ (question + answer, opens when clicked).</t>
+          <t>Order 14. Key: station_slug + place. The public "Buses &amp; taxis" section: a row with service or notes is listed in the table (Where / Service / Notes); a row with a photo also gets a photo card (photo_title, or place, + photo_caption). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Buses &amp; taxis.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>day_trips</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
+          <t>top_picks</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>15</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Order 16. Key: station_slug + name. One row per place under "Day trips": travel_time (e.g. ≈ 25–40 min) · transport (e.g. JR lines, direct), description, map_url (the Map button). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Day trips.</t>
+          <t>Order 15. Key: slug. The PLACES catalog (Admin &gt; Places): one record per place, used by every station. kind = grey line (e.g. Garden), category: landmark/food/shopping/museum/park/temple/daytrip/transport/help, entry_fee = cost, notes = visitor notes shown in the map popup. Day trips, transport and help items are places too (category daytrip / transport / help). Photos: Admin &gt; Places.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>buses_taxis</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
+          <t>station_places</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>16</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Order 18. Key: station_slug + place. The public "Buses &amp; taxis" section: a row with service or notes is listed in the table (Where / Service / Notes); a row with a photo also gets a photo card (photo_title, or place, + photo_caption). Photos cannot be uploaded here: add them in Admin &gt; Stations &gt; Buses &amp; taxis.</t>
+          <t>Order 16. Key: station_slug + top_pick_slug. ONE table for a place on a station. Common: exit_name (from exits sheet), walking_minutes, location (+ _japanese) free text, sort_order. Then 4 flags (1 = show there, 0 = not): is_top_pick = website main page / map popup (top_text = popup text, empty = the place's notes; top_caption = image caption; location_type inside/outside/inside_outside); is_thing = station page Things to do (thing_text = text, empty = place description; thing_caption = image caption); is_which_exit = Which exit? (needs exit_name; exit_note = note next to the exit; other_exits = more exit names separated by |); is_day_trip = Day trips (travel_time, transport). Every _japanese column is the Japanese version. At least one flag must be 1.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>top_picks</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
+          <t>hotels</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>17</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Order 20. Key: slug. The PLACES catalog (Admin &gt; Places): one record per place, used by both lists below. kind = grey line (e.g. Garden), category: landmark/food/shopping/museum/park/temple, entry_fee = cost. Photos: Admin &gt; Places.</t>
+          <t>Order 17. Key: slug. A hotel record (like top_picks): grey line = kind; map_url = Map button; booking_url = the "Check prices" button (Booking.com link; empty hides it). Photos: Admin &gt; Hotels.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>station_top_picks</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
+          <t>restaurants</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>18</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Order 21. Key: station_slug + top_pick_slug. TOP PICKS = the website main page / map popup. Picks a place for a station: exit_name (from exits sheet), walking_minutes, location_type inside/outside/inside_outside, location (+ _japanese) free text, sort_order.</t>
+          <t>Order 18. Key: slug. A restaurant record: grey line = kind; map_url = Map button. The note above the list is the stations column restaurants_note (**text** = bold). Photos: Admin &gt; Restaurants.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>station_things</t>
+          <t>station_hotels</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Order 21. Key: station_slug + top_pick_slug. THINGS TO DO = the station page (and "Which exit?"). A separate list from station_top_picks: picks a place from top_picks for this station: exit_name, walking_minutes, location (+ _japanese) free text, sort_order.</t>
+          <t>Order 19. Key: station_slug + hotel_slug. exit_name (from exits sheet), walking_minutes, location (free text), sort_order. Shown in Hotels and in Which exit?.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>hotels</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
+          <t>station_restaurants</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>20</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Order 22. Key: slug. A hotel record (like top_picks): grey line = kind; map_url = Map button; booking_url = the "Check prices" button (Booking.com link; empty hides it). Photos: Admin &gt; Hotels.</t>
+          <t>Order 20. Key: station_slug + restaurant_slug. exit_name (from exits sheet), walking_minutes, location (free text), sort_order. Shown in Restaurants and in Which exit?.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>restaurants</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Order 23. Key: slug. A restaurant record: grey line = kind; map_url = Map button. The note above the list is the stations column restaurants_note (**text** = bold). Photos: Admin &gt; Restaurants.</t>
-        </is>
-      </c>
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>station_hotels</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Order 24. Key: station_slug + hotel_slug. exit_name (from exits sheet), walking_minutes, location (free text), sort_order. Shown in Hotels and in Which exit?.</t>
-        </is>
-      </c>
+          <t>New columns (all optional - delete the column to leave stored values untouched):</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>station_restaurants</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Order 25. Key: station_slug + restaurant_slug. exit_name (from exits sheet), walking_minutes, location (free text), sort_order. Shown in Restaurants and in Which exit?.</t>
-        </is>
-      </c>
+          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
+        </is>
+      </c>
       <c r="B34" s="2" t="n"/>
       <c r="C34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>New columns (all optional - delete the column to leave stored values untouched):</t>
+          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
         </is>
       </c>
       <c r="B35" s="2" t="n"/>
@@ -1133,14 +1071,14 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>stations: region (e.g. 'Chiyoda City · Tokyo'), address (shown in the Overview facts card), stat_lines_note, stat_riders_value/_note, stat_opened_value/_note (+ _japanese). The 'N lines' number is automatic. A blank value hides that stat card.</t>
+          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>platforms: platform_number like '1・2' or '3/4' is drawn as stacked numbers; platform_group (e.g. 'Deep underground') puts platforms into a separate diagram; blank = main diagram. The strip colour comes from the line colour.</t>
+          <t>sides: 'exits' = exit names of this side, separated by | (they appear as tabs/chips in "Which exit?"; a side with no exits lists all). station_places: the places in "Which exit?" (is_which_exit = 1) - see its row above. The "Full station map" button uses the operator's website_url from the operators sheet.</t>
         </is>
       </c>
       <c r="B37" s="2" t="n"/>
@@ -1149,51 +1087,39 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>floor_facilities: 'exits' = nearby exit names separated by ; or , (exit names must exist in the exits sheet).</t>
+          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>sides: 'Sides of the station' on the public page. stations.sides_note / sides_note_japanese = the note about crossing between the sides. Train lines need no sheet: they come from lines + platforms.</t>
+          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>sides: 'exits' = exit names of this side, separated by | (they appear as tabs/chips in "Which exit?"; a side with no exits lists all). exit_places: the places in "Which exit?" - see its row above. The "Full station map" button uses the operator's website_url from the operators sheet.</t>
+          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>facilities: not part of the import. Add or change facilities (names, icons, group) in Admin &gt; Facilities; floor_facilities then uses their slugs.</t>
+          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>routes: 'Getting there' table on the public page (From / Route / Time / Cost). stations.routes_note / routes_note_japanese = the footnote under it.</t>
-        </is>
-      </c>
+      <c r="A42" s="2" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>tips: bullets under 'Exits &amp; station tips'. stations.exits_note / exits_note_japanese = the footnote under the exits table. Exit photos are NOT imported: upload them in Admin &gt; Stations &gt; Manage Exits (edit an exit &gt; Photo); exits.photo_caption / photo_caption_japanese is the text under the photo.</t>
-        </is>
-      </c>
+      <c r="A43" s="2" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>seasons: 'When to visit' on the public page, 2 columns (Spring/Summer/Autumn/Winter title is automatic). months e.g. 'Mar – May'; description is the text under it.</t>
-        </is>
-      </c>
+      <c r="A44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n"/>
@@ -1335,101 +1261,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="62" customWidth="1" min="6" max="6"/>
-    <col width="62" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>station_slug</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>name_japanese</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>sort_order</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>exits</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>exit_notes_japanese</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>#tokyo</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>KITTE &amp; KITTE Garden</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>KITTE・KITTEガーデン</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>sights</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>Marunouchi South Exit=1 min|Marunouchi Underground North Exit=underground</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
-        <is>
-          <t>Marunouchi South Exit=徒歩1分|Marunouchi Underground North Exit=地下直結</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1552,7 +1383,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1625,7 +1456,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1711,7 +1542,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1798,146 +1629,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="50" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>station_slug</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>name_japanese</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>travel_time</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>travel_time_japanese</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>transport</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>transport_japanese</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="I1" s="5" t="inlineStr">
-        <is>
-          <t>description_japanese</t>
-        </is>
-      </c>
-      <c r="J1" s="5" t="inlineStr">
-        <is>
-          <t>map_url</t>
-        </is>
-      </c>
-      <c r="K1" s="5" t="inlineStr">
-        <is>
-          <t>sort_order</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>#tokyo</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>Yokohama</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>横浜</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>≈ 25–40 min</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>約25〜40分</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>JR lines, direct</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
-        <is>
-          <t>JR線・乗換なし</t>
-        </is>
-      </c>
-      <c r="H2" s="7" t="inlineStr">
-        <is>
-          <t>GO TOKYO lists 25–40 minutes from Tokyo Station to Yokohama Station on JR lines; Yokohama's official visitors guide names the JR Tokaido, Yokosuka and Keihin-Tohoku lines.</t>
-        </is>
-      </c>
-      <c r="I2" s="7" t="inlineStr">
-        <is>
-          <t>東京駅から横浜駅までJR線で約25〜40分。東海道線・横須賀線・京浜東北線が利用できます。</t>
-        </is>
-      </c>
-      <c r="J2" s="7" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Yokohama+Station</t>
-        </is>
-      </c>
-      <c r="K2" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2071,7 +1763,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2216,6 +1908,359 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AA2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="18" customWidth="1" min="27" max="27"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>station_slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>top_pick_slug</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>exit_name</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>walking_minutes</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>location_japanese</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>location_type</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>is_top_pick</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>top_text</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>top_text_japanese</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>top_caption</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>top_caption_japanese</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>is_thing</t>
+        </is>
+      </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>thing_text</t>
+        </is>
+      </c>
+      <c r="P1" s="5" t="inlineStr">
+        <is>
+          <t>thing_text_japanese</t>
+        </is>
+      </c>
+      <c r="Q1" s="5" t="inlineStr">
+        <is>
+          <t>thing_caption</t>
+        </is>
+      </c>
+      <c r="R1" s="5" t="inlineStr">
+        <is>
+          <t>thing_caption_japanese</t>
+        </is>
+      </c>
+      <c r="S1" s="5" t="inlineStr">
+        <is>
+          <t>is_which_exit</t>
+        </is>
+      </c>
+      <c r="T1" s="5" t="inlineStr">
+        <is>
+          <t>exit_note</t>
+        </is>
+      </c>
+      <c r="U1" s="5" t="inlineStr">
+        <is>
+          <t>exit_note_japanese</t>
+        </is>
+      </c>
+      <c r="V1" s="5" t="inlineStr">
+        <is>
+          <t>other_exits</t>
+        </is>
+      </c>
+      <c r="W1" s="5" t="inlineStr">
+        <is>
+          <t>is_day_trip</t>
+        </is>
+      </c>
+      <c r="X1" s="5" t="inlineStr">
+        <is>
+          <t>travel_time</t>
+        </is>
+      </c>
+      <c r="Y1" s="5" t="inlineStr">
+        <is>
+          <t>travel_time_japanese</t>
+        </is>
+      </c>
+      <c r="Z1" s="5" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="AA1" s="5" t="inlineStr">
+        <is>
+          <t>transport_japanese</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#example-station</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>example-sight</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="6" t="n"/>
+      <c r="G2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>outside</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="6" t="n"/>
+      <c r="L2" s="6" t="n"/>
+      <c r="M2" s="6" t="n"/>
+      <c r="N2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" s="6" t="n"/>
+      <c r="P2" s="6" t="n"/>
+      <c r="Q2" s="6" t="n"/>
+      <c r="R2" s="6" t="n"/>
+      <c r="S2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2" s="6" t="n"/>
+      <c r="U2" s="6" t="n"/>
+      <c r="V2" s="6" t="n"/>
+      <c r="W2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" s="6" t="n"/>
+      <c r="Y2" s="6" t="n"/>
+      <c r="Z2" s="6" t="n"/>
+      <c r="AA2" s="6" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>slug</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>name_japanese</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>kind_japanese</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>description_japanese</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>map_url</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>booking_url</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>#the-tokyo-station-hotel</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>The Tokyo Station Hotel</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>東京ステーションホテル</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>In the station building</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>駅舎内</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Hotel inside the red-brick Marunouchi station building; it opened on November 2, 1915, one year after the station.</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr"/>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=The+Tokyo+Station+Hotel</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>https://www.booking.com/searchresults.html?ss=The+Tokyo+Station+Hotel</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2225,96 +2270,99 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>station_slug</t>
+          <t>slug</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>top_pick_slug</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>exit_name</t>
+          <t>name_japanese</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>walking_minutes</t>
+          <t>kind</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>location_type</t>
+          <t>kind_japanese</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>description</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
-          <t>location_japanese</t>
+          <t>description_japanese</t>
         </is>
       </c>
       <c r="H1" s="5" t="inlineStr">
         <is>
-          <t>sort_order</t>
+          <t>map_url</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>#example-station</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>example-sight</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>outside</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="n"/>
-      <c r="G2" s="6" t="n"/>
-      <c r="H2" s="6" t="n">
-        <v>1</v>
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>#rokurinsha</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Rokurinsha</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>六厘舎</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Tsukemen</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>つけ麺</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>The best-known shop on Tokyo Ramen Street, for tsukemen: thick noodles dipped into a separate bowl of rich broth. Buy a ticket at the machine by the d…</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr"/>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Rokurinsha</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"inside,outside,inside_outside"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -2411,317 +2459,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>station_slug</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>top_pick_slug</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>exit_name</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>walking_minutes</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>location</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>location_japanese</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>sort_order</t>
-        </is>
-      </c>
-      <c r="H1" s="8" t="n"/>
-      <c r="I1" s="9" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>#example-station</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>example-sight</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="6" t="n"/>
-      <c r="G2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="10" t="n"/>
-      <c r="I2" s="9" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>slug</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>name_japanese</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>kind</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>kind_japanese</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>description_japanese</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>map_url</t>
-        </is>
-      </c>
-      <c r="I1" s="5" t="inlineStr">
-        <is>
-          <t>booking_url</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>#the-tokyo-station-hotel</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>The Tokyo Station Hotel</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>東京ステーションホテル</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>In the station building</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>駅舎内</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>Hotel inside the red-brick Marunouchi station building; it opened on November 2, 1915, one year after the station.</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr"/>
-      <c r="H2" s="7" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=The+Tokyo+Station+Hotel</t>
-        </is>
-      </c>
-      <c r="I2" s="7" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/searchresults.html?ss=The+Tokyo+Station+Hotel</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>slug</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>name_japanese</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>kind</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>kind_japanese</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>description_japanese</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>map_url</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>#rokurinsha</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>Rokurinsha</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>六厘舎</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>Tsukemen</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>つけ麺</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>The best-known shop on Tokyo Ramen Street, for tsukemen: thick noodles dipped into a separate bowl of rich broth. Buy a ticket at the machine by the d…</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr"/>
-      <c r="H2" s="7" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Rokurinsha</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2803,7 +2540,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Platform map: direction (left/right/north), legend colour categories, per-diagram note and line details; importer + template columns (migration 0050)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpccaTkeawAufrNzVaBTSd
</commit_message>
<xml_diff>
--- a/public/templates/tokyo-guide-bulk-upload-template.xlsx
+++ b/public/templates/tokyo-guide-bulk-upload-template.xlsx
@@ -768,7 +768,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Order 3. is_verified: 1 or 0. verified_at: YYYY-MM-DD.</t>
+          <t>Order 3. is_verified: 1 or 0. verified_at: YYYY-MM-DD. Platform map direction: platform_map_left / platform_map_right = the labels above the left / right of the map (e.g. Marunouchi · West), platform_map_north = 1 shows the N ↑ arrow (+ _japanese).</t>
         </is>
       </c>
     </row>
@@ -843,7 +843,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Order 8. Key: station_slug + platform_number + line_slug. line_slug and floor_name are optional.</t>
+          <t>Order 8. Key: station_slug + platform_number + line_slug. line_slug and floor_name are optional. MAP: platform_group (e.g. Deep underground) = a separate diagram, group_note = text beside its name (e.g. their own numbers 1–4). legend_label / legend_color = the colour key under the map (platforms with the same label share one row; empty = the line name and colour). Under a named diagram the map also lists "&lt;line&gt; platforms · &lt;floor_name&gt; · &lt;notes&gt;" (e.g. Sobu platforms · B5 · 230 m from Marunouchi North gate). Every _japanese column is the Japanese version.</t>
         </is>
       </c>
     </row>
@@ -2772,7 +2772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AI2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2805,6 +2805,11 @@
     <col width="36" customWidth="1" min="28" max="28"/>
     <col width="40" customWidth="1" min="29" max="29"/>
     <col width="40" customWidth="1" min="30" max="30"/>
+    <col width="22" customWidth="1" min="31" max="31"/>
+    <col width="22" customWidth="1" min="32" max="32"/>
+    <col width="22" customWidth="1" min="33" max="33"/>
+    <col width="22" customWidth="1" min="34" max="34"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2958,6 +2963,31 @@
           <t>restaurants_note_japanese</t>
         </is>
       </c>
+      <c r="AE1" s="5" t="inlineStr">
+        <is>
+          <t>platform_map_left</t>
+        </is>
+      </c>
+      <c r="AF1" s="5" t="inlineStr">
+        <is>
+          <t>platform_map_left_japanese</t>
+        </is>
+      </c>
+      <c r="AG1" s="5" t="inlineStr">
+        <is>
+          <t>platform_map_right</t>
+        </is>
+      </c>
+      <c r="AH1" s="5" t="inlineStr">
+        <is>
+          <t>platform_map_right_japanese</t>
+        </is>
+      </c>
+      <c r="AI1" s="5" t="inlineStr">
+        <is>
+          <t>platform_map_north</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -3099,6 +3129,29 @@
         <is>
           <t>駅構内の表示は「出口」、駅外の表示は「入口」ですが、同じ場所です。</t>
         </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Marunouchi · West</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>丸の内・西</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>Yaesu · East</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>八重洲・東</t>
+        </is>
+      </c>
+      <c r="AI2" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3541,7 +3594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3555,6 +3608,11 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3613,6 +3671,31 @@
           <t>platform_group_japanese</t>
         </is>
       </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>group_note</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>group_note_japanese</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>legend_label</t>
+        </is>
+      </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>legend_label_japanese</t>
+        </is>
+      </c>
+      <c r="P1" s="5" t="inlineStr">
+        <is>
+          <t>legend_color</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -3658,6 +3741,31 @@
       <c r="K2" s="6" t="inlineStr">
         <is>
           <t>地下深部</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>their own numbers 1–4</t>
+        </is>
+      </c>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
+          <t>それぞれ独自の番号1〜4</t>
+        </is>
+      </c>
+      <c r="N2" s="6" t="inlineStr">
+        <is>
+          <t>JR lines</t>
+        </is>
+      </c>
+      <c r="O2" s="6" t="inlineStr">
+        <is>
+          <t>JR線</t>
+        </is>
+      </c>
+      <c r="P2" s="6" t="inlineStr">
+        <is>
+          <t>#555555</t>
         </is>
       </c>
     </row>

</xml_diff>